<commit_message>
Only ever produce the template; delete the worked workbook
The download is now one button and one file: Financial Data and Sources filled,
Common-Size, Trend and Ratios carrying every label and heading with the analysis
cells empty. Deriving those is the point of handing someone the file.

This removes the capability rather than hiding the button. The formula-filled
template is deleted, build() takes no mode, and the xlsx endpoint ignores one --
?mode=full returns the same template. A URL that can be edited to hand back the
answers is a URL someone will edit.

data/template_data_only.xlsx is now data/template.xlsx, since there is only one.
The worked version stays in git history if it is ever wanted back.

/api/company/{ticker} keeps ?mode=data. It only affects the JSON and the
on-screen market multiples, never the workbook.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/template.xlsx
+++ b/data/template.xlsx
@@ -71,7 +71,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -108,11 +108,6 @@
         <fgColor rgb="002E5C8A"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE0E0"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -140,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -180,7 +175,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -568,9 +562,9 @@
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Generated by edgar-query. The Financial Data sheet is already filled from SEC EDGAR; every other sheet is live formulas.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Generated by edgar-query. The Financial Data sheet is filled from SEC EDGAR. Every other sheet is yours to build.</t>
         </is>
       </c>
     </row>
@@ -584,7 +578,7 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>One company. Five fiscal years. Statements, common-size, trend and ratios are all filled in and linked - every analysis cell is a live formula pointing at Financial Data.</t>
+          <t>One company. Five fiscal years. The statements are already in front of you. What you build is the analysis: common-size statements, a trend analysis, and a set of ratios.</t>
         </is>
       </c>
     </row>
@@ -621,7 +615,7 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Financial Data  -  Filled from SEC EDGAR. Every other sheet links back to it.</t>
+          <t xml:space="preserve">   Financial Data  -  Already filled from SEC EDGAR. Read it, check it, but do not retype it.</t>
         </is>
       </c>
     </row>
@@ -698,7 +692,7 @@
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Cross-check anything that looks wrong against the filing itself at sec.gov/edgar. Note that a single 10-K carries only TWO years of balance sheet data; the API aggregates across filings to reach five.</t>
+          <t>Cross-check anything that looks wrong against the filing itself at sec.gov/edgar. Interest Expense is already entered as a positive number, because it is a cost.</t>
         </is>
       </c>
     </row>
@@ -712,28 +706,28 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>1. INTEREST EXPENSE is usually shown as a NEGATIVE number on financial websites (-163.4). Type it in as a POSITIVE number (163.4). It is a cost, and the template already treats it as one. If you leave it negative, Times Interest Earned comes out negative and nothing downstream makes sense.</t>
+          <t>1. Point every formula at the Financial Data sheet, not at a number you copied out of it. That is the whole exercise - see 'The one rule about formulas' above.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>2. Your balance sheet total may be off by a few tenths. That is rounding in the published figures, not your mistake. Off by tens or hundreds IS your mistake.</t>
+          <t>2. Your balance sheet check row may be off by a few tenths. That is rounding in the published figures. Off by tens or hundreds means something is genuinely wrong - tell me.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Picking a company</t>
+          <t>About your company</t>
         </is>
       </c>
     </row>
     <row r="36" ht="56" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Pick a company you have heard of that makes or sells something physical. Avoid banks, insurers, and investment firms -- their balance sheets have no current assets subtotal and most of these ratios will not compute. Avoid companies that lost money in most of the five years; negative net income makes margins and returns hard to read.</t>
+          <t>Companies with a captive finance arm, and any bank or insurer, do not publish a current-assets subtotal, so the liquidity ratios cannot be computed for them. The tool refuses those up front, so whatever you were given works.</t>
         </is>
       </c>
     </row>
@@ -747,28 +741,28 @@
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   [ ]  The check row on the Financial Data sheet reads within about 1.0 of zero in all five years</t>
+          <t xml:space="preserve">   [ ]  Every green cell contains a formula, not a typed number</t>
         </is>
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   [ ]  Interest Expense is shown positive (it is a cost; the app already flips the sign)</t>
+          <t xml:space="preserve">   [ ]  Every formula points back to the Financial Data sheet</t>
         </is>
       </c>
     </row>
     <row r="41" ht="14" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   [ ]  Every green cell still contains a formula, not a pasted number</t>
+          <t xml:space="preserve">   [ ]  The DuPont check row on the Ratios sheet shows a difference of zero</t>
         </is>
       </c>
     </row>
     <row r="42" ht="14" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   [ ]  The DuPont check row on the Ratios sheet shows a difference of zero</t>
+          <t xml:space="preserve">   [ ]  The check row on the Financial Data sheet reads within about 1.0 of zero in all five years</t>
         </is>
       </c>
     </row>
@@ -1332,26 +1326,11 @@
           <t>Revenue (Net Sales)</t>
         </is>
       </c>
-      <c r="C10" s="16">
-        <f>'Financial Data'!C10/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D10" s="16">
-        <f>'Financial Data'!D10/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E10" s="16">
-        <f>'Financial Data'!E10/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F10" s="16">
-        <f>'Financial Data'!F10/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G10" s="16">
-        <f>'Financial Data'!G10/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="16" t="n"/>
+      <c r="G10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1359,26 +1338,11 @@
           <t>Cost of Revenue (COGS)</t>
         </is>
       </c>
-      <c r="C11" s="16">
-        <f>'Financial Data'!C11/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D11" s="16">
-        <f>'Financial Data'!D11/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E11" s="16">
-        <f>'Financial Data'!E11/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F11" s="16">
-        <f>'Financial Data'!F11/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G11" s="16">
-        <f>'Financial Data'!G11/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -1386,26 +1350,11 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="C12" s="16">
-        <f>'Financial Data'!C12/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D12" s="16">
-        <f>'Financial Data'!D12/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E12" s="16">
-        <f>'Financial Data'!E12/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F12" s="16">
-        <f>'Financial Data'!F12/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G12" s="16">
-        <f>'Financial Data'!G12/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C12" s="16" t="n"/>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="16" t="n"/>
+      <c r="G12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1413,26 +1362,11 @@
           <t>Operating Expenses</t>
         </is>
       </c>
-      <c r="C13" s="16">
-        <f>'Financial Data'!C13/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D13" s="16">
-        <f>'Financial Data'!D13/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E13" s="16">
-        <f>'Financial Data'!E13/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F13" s="16">
-        <f>'Financial Data'!F13/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G13" s="16">
-        <f>'Financial Data'!G13/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C13" s="16" t="n"/>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1440,26 +1374,11 @@
           <t>Operating Income (EBIT)</t>
         </is>
       </c>
-      <c r="C14" s="16">
-        <f>'Financial Data'!C14/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D14" s="16">
-        <f>'Financial Data'!D14/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E14" s="16">
-        <f>'Financial Data'!E14/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F14" s="16">
-        <f>'Financial Data'!F14/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G14" s="16">
-        <f>'Financial Data'!G14/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="16" t="n"/>
+      <c r="G14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1467,26 +1386,11 @@
           <t>Interest Expense</t>
         </is>
       </c>
-      <c r="C15" s="16">
-        <f>'Financial Data'!C15/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D15" s="16">
-        <f>'Financial Data'!D15/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E15" s="16">
-        <f>'Financial Data'!E15/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F15" s="16">
-        <f>'Financial Data'!F15/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G15" s="16">
-        <f>'Financial Data'!G15/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="16" t="n"/>
+      <c r="G15" s="16" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1494,26 +1398,11 @@
           <t>Pretax Income</t>
         </is>
       </c>
-      <c r="C16" s="16">
-        <f>'Financial Data'!C16/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D16" s="16">
-        <f>'Financial Data'!D16/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E16" s="16">
-        <f>'Financial Data'!E16/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F16" s="16">
-        <f>'Financial Data'!F16/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G16" s="16">
-        <f>'Financial Data'!G16/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
+      <c r="G16" s="16" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1521,26 +1410,11 @@
           <t>Income Tax Expense</t>
         </is>
       </c>
-      <c r="C17" s="16">
-        <f>'Financial Data'!C17/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D17" s="16">
-        <f>'Financial Data'!D17/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E17" s="16">
-        <f>'Financial Data'!E17/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F17" s="16">
-        <f>'Financial Data'!F17/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G17" s="16">
-        <f>'Financial Data'!G17/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="16" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1548,26 +1422,11 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="C18" s="16">
-        <f>'Financial Data'!C18/'Financial Data'!C$10</f>
-        <v/>
-      </c>
-      <c r="D18" s="16">
-        <f>'Financial Data'!D18/'Financial Data'!D$10</f>
-        <v/>
-      </c>
-      <c r="E18" s="16">
-        <f>'Financial Data'!E18/'Financial Data'!E$10</f>
-        <v/>
-      </c>
-      <c r="F18" s="16">
-        <f>'Financial Data'!F18/'Financial Data'!F$10</f>
-        <v/>
-      </c>
-      <c r="G18" s="16">
-        <f>'Financial Data'!G18/'Financial Data'!G$10</f>
-        <v/>
-      </c>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="16" t="n"/>
+      <c r="G18" s="16" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -1587,26 +1446,11 @@
           <t>Cash &amp; Short-Term Investments</t>
         </is>
       </c>
-      <c r="C21" s="16">
-        <f>'Financial Data'!C21/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D21" s="16">
-        <f>'Financial Data'!D21/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E21" s="16">
-        <f>'Financial Data'!E21/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F21" s="16">
-        <f>'Financial Data'!F21/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G21" s="16">
-        <f>'Financial Data'!G21/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="16" t="n"/>
+      <c r="G21" s="16" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1614,26 +1458,11 @@
           <t>Accounts Receivable</t>
         </is>
       </c>
-      <c r="C22" s="16">
-        <f>'Financial Data'!C22/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D22" s="16">
-        <f>'Financial Data'!D22/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E22" s="16">
-        <f>'Financial Data'!E22/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F22" s="16">
-        <f>'Financial Data'!F22/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G22" s="16">
-        <f>'Financial Data'!G22/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="n"/>
+      <c r="G22" s="16" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1641,26 +1470,11 @@
           <t>Inventory</t>
         </is>
       </c>
-      <c r="C23" s="16">
-        <f>'Financial Data'!C23/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D23" s="16">
-        <f>'Financial Data'!D23/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E23" s="16">
-        <f>'Financial Data'!E23/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F23" s="16">
-        <f>'Financial Data'!F23/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G23" s="16">
-        <f>'Financial Data'!G23/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="n"/>
+      <c r="G23" s="16" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1668,26 +1482,11 @@
           <t>Other Current Assets</t>
         </is>
       </c>
-      <c r="C24" s="16">
-        <f>'Financial Data'!C24/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D24" s="16">
-        <f>'Financial Data'!D24/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E24" s="16">
-        <f>'Financial Data'!E24/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F24" s="16">
-        <f>'Financial Data'!F24/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G24" s="16">
-        <f>'Financial Data'!G24/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="16" t="n"/>
+      <c r="G24" s="16" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1695,26 +1494,11 @@
           <t>Total Current Assets</t>
         </is>
       </c>
-      <c r="C25" s="16">
-        <f>'Financial Data'!C25/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D25" s="16">
-        <f>'Financial Data'!D25/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E25" s="16">
-        <f>'Financial Data'!E25/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F25" s="16">
-        <f>'Financial Data'!F25/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G25" s="16">
-        <f>'Financial Data'!G25/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="16" t="n"/>
+      <c r="G25" s="16" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1722,26 +1506,11 @@
           <t>Property, Plant &amp; Equipment (net)</t>
         </is>
       </c>
-      <c r="C26" s="16">
-        <f>'Financial Data'!C26/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D26" s="16">
-        <f>'Financial Data'!D26/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E26" s="16">
-        <f>'Financial Data'!E26/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F26" s="16">
-        <f>'Financial Data'!F26/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G26" s="16">
-        <f>'Financial Data'!G26/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="16" t="n"/>
+      <c r="G26" s="16" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1749,26 +1518,11 @@
           <t>Goodwill &amp; Intangible Assets</t>
         </is>
       </c>
-      <c r="C27" s="16">
-        <f>'Financial Data'!C27/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D27" s="16">
-        <f>'Financial Data'!D27/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E27" s="16">
-        <f>'Financial Data'!E27/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F27" s="16">
-        <f>'Financial Data'!F27/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
-        <f>'Financial Data'!G27/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="16" t="n"/>
+      <c r="G27" s="16" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1776,26 +1530,11 @@
           <t>Other Long-Term Assets</t>
         </is>
       </c>
-      <c r="C28" s="16">
-        <f>'Financial Data'!C28/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D28" s="16">
-        <f>'Financial Data'!D28/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E28" s="16">
-        <f>'Financial Data'!E28/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F28" s="16">
-        <f>'Financial Data'!F28/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G28" s="16">
-        <f>'Financial Data'!G28/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="16" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1803,26 +1542,11 @@
           <t>Total Assets</t>
         </is>
       </c>
-      <c r="C29" s="16">
-        <f>'Financial Data'!C29/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D29" s="16">
-        <f>'Financial Data'!D29/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E29" s="16">
-        <f>'Financial Data'!E29/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F29" s="16">
-        <f>'Financial Data'!F29/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G29" s="16">
-        <f>'Financial Data'!G29/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="n"/>
+      <c r="G29" s="16" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
@@ -1837,26 +1561,11 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="C32" s="16">
-        <f>'Financial Data'!C32/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D32" s="16">
-        <f>'Financial Data'!D32/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E32" s="16">
-        <f>'Financial Data'!E32/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F32" s="16">
-        <f>'Financial Data'!F32/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G32" s="16">
-        <f>'Financial Data'!G32/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="16" t="n"/>
+      <c r="E32" s="16" t="n"/>
+      <c r="F32" s="16" t="n"/>
+      <c r="G32" s="16" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -1864,26 +1573,11 @@
           <t>Short-Term Debt &amp; Current Portion of LTD</t>
         </is>
       </c>
-      <c r="C33" s="16">
-        <f>'Financial Data'!C33/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D33" s="16">
-        <f>'Financial Data'!D33/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E33" s="16">
-        <f>'Financial Data'!E33/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F33" s="16">
-        <f>'Financial Data'!F33/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G33" s="16">
-        <f>'Financial Data'!G33/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C33" s="16" t="n"/>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="16" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -1891,26 +1585,11 @@
           <t>Other Current Liabilities</t>
         </is>
       </c>
-      <c r="C34" s="16">
-        <f>'Financial Data'!C34/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D34" s="16">
-        <f>'Financial Data'!D34/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E34" s="16">
-        <f>'Financial Data'!E34/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F34" s="16">
-        <f>'Financial Data'!F34/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G34" s="16">
-        <f>'Financial Data'!G34/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C34" s="16" t="n"/>
+      <c r="D34" s="16" t="n"/>
+      <c r="E34" s="16" t="n"/>
+      <c r="F34" s="16" t="n"/>
+      <c r="G34" s="16" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -1918,26 +1597,11 @@
           <t>Total Current Liabilities</t>
         </is>
       </c>
-      <c r="C35" s="16">
-        <f>'Financial Data'!C35/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D35" s="16">
-        <f>'Financial Data'!D35/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E35" s="16">
-        <f>'Financial Data'!E35/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F35" s="16">
-        <f>'Financial Data'!F35/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G35" s="16">
-        <f>'Financial Data'!G35/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C35" s="16" t="n"/>
+      <c r="D35" s="16" t="n"/>
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="16" t="n"/>
+      <c r="G35" s="16" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1945,26 +1609,11 @@
           <t>Long-Term Debt</t>
         </is>
       </c>
-      <c r="C36" s="16">
-        <f>'Financial Data'!C36/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D36" s="16">
-        <f>'Financial Data'!D36/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E36" s="16">
-        <f>'Financial Data'!E36/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F36" s="16">
-        <f>'Financial Data'!F36/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G36" s="16">
-        <f>'Financial Data'!G36/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C36" s="16" t="n"/>
+      <c r="D36" s="16" t="n"/>
+      <c r="E36" s="16" t="n"/>
+      <c r="F36" s="16" t="n"/>
+      <c r="G36" s="16" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -1972,26 +1621,11 @@
           <t>Other Long-Term Liabilities</t>
         </is>
       </c>
-      <c r="C37" s="16">
-        <f>'Financial Data'!C37/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D37" s="16">
-        <f>'Financial Data'!D37/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E37" s="16">
-        <f>'Financial Data'!E37/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F37" s="16">
-        <f>'Financial Data'!F37/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G37" s="16">
-        <f>'Financial Data'!G37/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C37" s="16" t="n"/>
+      <c r="D37" s="16" t="n"/>
+      <c r="E37" s="16" t="n"/>
+      <c r="F37" s="16" t="n"/>
+      <c r="G37" s="16" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -1999,26 +1633,11 @@
           <t>Total Liabilities</t>
         </is>
       </c>
-      <c r="C38" s="16">
-        <f>'Financial Data'!C38/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D38" s="16">
-        <f>'Financial Data'!D38/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E38" s="16">
-        <f>'Financial Data'!E38/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F38" s="16">
-        <f>'Financial Data'!F38/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G38" s="16">
-        <f>'Financial Data'!G38/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C38" s="16" t="n"/>
+      <c r="D38" s="16" t="n"/>
+      <c r="E38" s="16" t="n"/>
+      <c r="F38" s="16" t="n"/>
+      <c r="G38" s="16" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -2026,26 +1645,11 @@
           <t>Total Shareholders' Equity</t>
         </is>
       </c>
-      <c r="C39" s="16">
-        <f>'Financial Data'!C39/'Financial Data'!C$29</f>
-        <v/>
-      </c>
-      <c r="D39" s="16">
-        <f>'Financial Data'!D39/'Financial Data'!D$29</f>
-        <v/>
-      </c>
-      <c r="E39" s="16">
-        <f>'Financial Data'!E39/'Financial Data'!E$29</f>
-        <v/>
-      </c>
-      <c r="F39" s="16">
-        <f>'Financial Data'!F39/'Financial Data'!F$29</f>
-        <v/>
-      </c>
-      <c r="G39" s="16">
-        <f>'Financial Data'!G39/'Financial Data'!G$29</f>
-        <v/>
-      </c>
+      <c r="C39" s="16" t="n"/>
+      <c r="D39" s="16" t="n"/>
+      <c r="E39" s="16" t="n"/>
+      <c r="F39" s="16" t="n"/>
+      <c r="G39" s="16" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2144,22 +1748,10 @@
         </is>
       </c>
       <c r="C6" s="20" t="n"/>
-      <c r="D6" s="16">
-        <f>('Financial Data'!D10-'Financial Data'!C10)/'Financial Data'!C10</f>
-        <v/>
-      </c>
-      <c r="E6" s="16">
-        <f>('Financial Data'!E10-'Financial Data'!D10)/'Financial Data'!D10</f>
-        <v/>
-      </c>
-      <c r="F6" s="16">
-        <f>('Financial Data'!F10-'Financial Data'!E10)/'Financial Data'!E10</f>
-        <v/>
-      </c>
-      <c r="G6" s="16">
-        <f>('Financial Data'!G10-'Financial Data'!F10)/'Financial Data'!F10</f>
-        <v/>
-      </c>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="16" t="n"/>
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="16" t="n"/>
       <c r="I6" s="11" t="inlineStr">
         <is>
           <t>(This year - Last year) / Last year. There is no percent change for your earliest year because there is nothing before it.</t>
@@ -2173,22 +1765,10 @@
         </is>
       </c>
       <c r="C7" s="20" t="n"/>
-      <c r="D7" s="16">
-        <f>('Financial Data'!D11-'Financial Data'!C11)/'Financial Data'!C11</f>
-        <v/>
-      </c>
-      <c r="E7" s="16">
-        <f>('Financial Data'!E11-'Financial Data'!D11)/'Financial Data'!D11</f>
-        <v/>
-      </c>
-      <c r="F7" s="16">
-        <f>('Financial Data'!F11-'Financial Data'!E11)/'Financial Data'!E11</f>
-        <v/>
-      </c>
-      <c r="G7" s="16">
-        <f>('Financial Data'!G11-'Financial Data'!F11)/'Financial Data'!F11</f>
-        <v/>
-      </c>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2197,22 +1777,10 @@
         </is>
       </c>
       <c r="C8" s="20" t="n"/>
-      <c r="D8" s="16">
-        <f>('Financial Data'!D12-'Financial Data'!C12)/'Financial Data'!C12</f>
-        <v/>
-      </c>
-      <c r="E8" s="16">
-        <f>('Financial Data'!E12-'Financial Data'!D12)/'Financial Data'!D12</f>
-        <v/>
-      </c>
-      <c r="F8" s="16">
-        <f>('Financial Data'!F12-'Financial Data'!E12)/'Financial Data'!E12</f>
-        <v/>
-      </c>
-      <c r="G8" s="16">
-        <f>('Financial Data'!G12-'Financial Data'!F12)/'Financial Data'!F12</f>
-        <v/>
-      </c>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="16" t="n"/>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="16" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2221,22 +1789,10 @@
         </is>
       </c>
       <c r="C9" s="20" t="n"/>
-      <c r="D9" s="16">
-        <f>('Financial Data'!D14-'Financial Data'!C14)/'Financial Data'!C14</f>
-        <v/>
-      </c>
-      <c r="E9" s="16">
-        <f>('Financial Data'!E14-'Financial Data'!D14)/'Financial Data'!D14</f>
-        <v/>
-      </c>
-      <c r="F9" s="16">
-        <f>('Financial Data'!F14-'Financial Data'!E14)/'Financial Data'!E14</f>
-        <v/>
-      </c>
-      <c r="G9" s="16">
-        <f>('Financial Data'!G14-'Financial Data'!F14)/'Financial Data'!F14</f>
-        <v/>
-      </c>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="16" t="n"/>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="16" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2245,22 +1801,10 @@
         </is>
       </c>
       <c r="C10" s="20" t="n"/>
-      <c r="D10" s="16">
-        <f>('Financial Data'!D18-'Financial Data'!C18)/'Financial Data'!C18</f>
-        <v/>
-      </c>
-      <c r="E10" s="16">
-        <f>('Financial Data'!E18-'Financial Data'!D18)/'Financial Data'!D18</f>
-        <v/>
-      </c>
-      <c r="F10" s="16">
-        <f>('Financial Data'!F18-'Financial Data'!E18)/'Financial Data'!E18</f>
-        <v/>
-      </c>
-      <c r="G10" s="16">
-        <f>('Financial Data'!G18-'Financial Data'!F18)/'Financial Data'!F18</f>
-        <v/>
-      </c>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="16" t="n"/>
+      <c r="G10" s="16" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2269,22 +1813,10 @@
         </is>
       </c>
       <c r="C11" s="20" t="n"/>
-      <c r="D11" s="16">
-        <f>('Financial Data'!D23-'Financial Data'!C23)/'Financial Data'!C23</f>
-        <v/>
-      </c>
-      <c r="E11" s="16">
-        <f>('Financial Data'!E23-'Financial Data'!D23)/'Financial Data'!D23</f>
-        <v/>
-      </c>
-      <c r="F11" s="16">
-        <f>('Financial Data'!F23-'Financial Data'!E23)/'Financial Data'!E23</f>
-        <v/>
-      </c>
-      <c r="G11" s="16">
-        <f>('Financial Data'!G23-'Financial Data'!F23)/'Financial Data'!F23</f>
-        <v/>
-      </c>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2293,22 +1825,10 @@
         </is>
       </c>
       <c r="C12" s="20" t="n"/>
-      <c r="D12" s="16">
-        <f>('Financial Data'!D25-'Financial Data'!C25)/'Financial Data'!C25</f>
-        <v/>
-      </c>
-      <c r="E12" s="16">
-        <f>('Financial Data'!E25-'Financial Data'!D25)/'Financial Data'!D25</f>
-        <v/>
-      </c>
-      <c r="F12" s="16">
-        <f>('Financial Data'!F25-'Financial Data'!E25)/'Financial Data'!E25</f>
-        <v/>
-      </c>
-      <c r="G12" s="16">
-        <f>('Financial Data'!G25-'Financial Data'!F25)/'Financial Data'!F25</f>
-        <v/>
-      </c>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="16" t="n"/>
+      <c r="G12" s="16" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2317,22 +1837,10 @@
         </is>
       </c>
       <c r="C13" s="20" t="n"/>
-      <c r="D13" s="16">
-        <f>('Financial Data'!D29-'Financial Data'!C29)/'Financial Data'!C29</f>
-        <v/>
-      </c>
-      <c r="E13" s="16">
-        <f>('Financial Data'!E29-'Financial Data'!D29)/'Financial Data'!D29</f>
-        <v/>
-      </c>
-      <c r="F13" s="16">
-        <f>('Financial Data'!F29-'Financial Data'!E29)/'Financial Data'!E29</f>
-        <v/>
-      </c>
-      <c r="G13" s="16">
-        <f>('Financial Data'!G29-'Financial Data'!F29)/'Financial Data'!F29</f>
-        <v/>
-      </c>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="16" t="n"/>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="16" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -2341,22 +1849,10 @@
         </is>
       </c>
       <c r="C14" s="20" t="n"/>
-      <c r="D14" s="16">
-        <f>('Financial Data'!D38-'Financial Data'!C38)/'Financial Data'!C38</f>
-        <v/>
-      </c>
-      <c r="E14" s="16">
-        <f>('Financial Data'!E38-'Financial Data'!D38)/'Financial Data'!D38</f>
-        <v/>
-      </c>
-      <c r="F14" s="16">
-        <f>('Financial Data'!F38-'Financial Data'!E38)/'Financial Data'!E38</f>
-        <v/>
-      </c>
-      <c r="G14" s="16">
-        <f>('Financial Data'!G38-'Financial Data'!F38)/'Financial Data'!F38</f>
-        <v/>
-      </c>
+      <c r="D14" s="16" t="n"/>
+      <c r="E14" s="16" t="n"/>
+      <c r="F14" s="16" t="n"/>
+      <c r="G14" s="16" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -2365,22 +1861,10 @@
         </is>
       </c>
       <c r="C15" s="20" t="n"/>
-      <c r="D15" s="16">
-        <f>('Financial Data'!D39-'Financial Data'!C39)/'Financial Data'!C39</f>
-        <v/>
-      </c>
-      <c r="E15" s="16">
-        <f>('Financial Data'!E39-'Financial Data'!D39)/'Financial Data'!D39</f>
-        <v/>
-      </c>
-      <c r="F15" s="16">
-        <f>('Financial Data'!F39-'Financial Data'!E39)/'Financial Data'!E39</f>
-        <v/>
-      </c>
-      <c r="G15" s="16">
-        <f>('Financial Data'!G39-'Financial Data'!F39)/'Financial Data'!F39</f>
-        <v/>
-      </c>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="16" t="n"/>
+      <c r="G15" s="16" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -2430,26 +1914,11 @@
           <t>Revenue (Net Sales)</t>
         </is>
       </c>
-      <c r="C20" s="21">
-        <f>'Financial Data'!C10/'Financial Data'!$C$10*100</f>
-        <v/>
-      </c>
-      <c r="D20" s="21">
-        <f>'Financial Data'!D10/'Financial Data'!$C$10*100</f>
-        <v/>
-      </c>
-      <c r="E20" s="21">
-        <f>'Financial Data'!E10/'Financial Data'!$C$10*100</f>
-        <v/>
-      </c>
-      <c r="F20" s="21">
-        <f>'Financial Data'!F10/'Financial Data'!$C$10*100</f>
-        <v/>
-      </c>
-      <c r="G20" s="21">
-        <f>'Financial Data'!G10/'Financial Data'!$C$10*100</f>
-        <v/>
-      </c>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="21" t="n"/>
+      <c r="G20" s="21" t="n"/>
       <c r="I20" s="11" t="inlineStr">
         <is>
           <t>Year N / earliest year x 100. Your earliest year will come out to exactly 100.0 - that is the check that you did it right. Lock the base year column with $.</t>
@@ -2462,26 +1931,11 @@
           <t>Cost of Revenue (COGS)</t>
         </is>
       </c>
-      <c r="C21" s="21">
-        <f>'Financial Data'!C11/'Financial Data'!$C$11*100</f>
-        <v/>
-      </c>
-      <c r="D21" s="21">
-        <f>'Financial Data'!D11/'Financial Data'!$C$11*100</f>
-        <v/>
-      </c>
-      <c r="E21" s="21">
-        <f>'Financial Data'!E11/'Financial Data'!$C$11*100</f>
-        <v/>
-      </c>
-      <c r="F21" s="21">
-        <f>'Financial Data'!F11/'Financial Data'!$C$11*100</f>
-        <v/>
-      </c>
-      <c r="G21" s="21">
-        <f>'Financial Data'!G11/'Financial Data'!$C$11*100</f>
-        <v/>
-      </c>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="21" t="n"/>
+      <c r="G21" s="21" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -2489,26 +1943,11 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="C22" s="21">
-        <f>'Financial Data'!C12/'Financial Data'!$C$12*100</f>
-        <v/>
-      </c>
-      <c r="D22" s="21">
-        <f>'Financial Data'!D12/'Financial Data'!$C$12*100</f>
-        <v/>
-      </c>
-      <c r="E22" s="21">
-        <f>'Financial Data'!E12/'Financial Data'!$C$12*100</f>
-        <v/>
-      </c>
-      <c r="F22" s="21">
-        <f>'Financial Data'!F12/'Financial Data'!$C$12*100</f>
-        <v/>
-      </c>
-      <c r="G22" s="21">
-        <f>'Financial Data'!G12/'Financial Data'!$C$12*100</f>
-        <v/>
-      </c>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="21" t="n"/>
+      <c r="E22" s="21" t="n"/>
+      <c r="F22" s="21" t="n"/>
+      <c r="G22" s="21" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -2516,26 +1955,11 @@
           <t>Operating Income (EBIT)</t>
         </is>
       </c>
-      <c r="C23" s="21">
-        <f>'Financial Data'!C14/'Financial Data'!$C$14*100</f>
-        <v/>
-      </c>
-      <c r="D23" s="21">
-        <f>'Financial Data'!D14/'Financial Data'!$C$14*100</f>
-        <v/>
-      </c>
-      <c r="E23" s="21">
-        <f>'Financial Data'!E14/'Financial Data'!$C$14*100</f>
-        <v/>
-      </c>
-      <c r="F23" s="21">
-        <f>'Financial Data'!F14/'Financial Data'!$C$14*100</f>
-        <v/>
-      </c>
-      <c r="G23" s="21">
-        <f>'Financial Data'!G14/'Financial Data'!$C$14*100</f>
-        <v/>
-      </c>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -2543,26 +1967,11 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="C24" s="21">
-        <f>'Financial Data'!C18/'Financial Data'!$C$18*100</f>
-        <v/>
-      </c>
-      <c r="D24" s="21">
-        <f>'Financial Data'!D18/'Financial Data'!$C$18*100</f>
-        <v/>
-      </c>
-      <c r="E24" s="21">
-        <f>'Financial Data'!E18/'Financial Data'!$C$18*100</f>
-        <v/>
-      </c>
-      <c r="F24" s="21">
-        <f>'Financial Data'!F18/'Financial Data'!$C$18*100</f>
-        <v/>
-      </c>
-      <c r="G24" s="21">
-        <f>'Financial Data'!G18/'Financial Data'!$C$18*100</f>
-        <v/>
-      </c>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
+      <c r="E24" s="21" t="n"/>
+      <c r="F24" s="21" t="n"/>
+      <c r="G24" s="21" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -2570,26 +1979,11 @@
           <t>Inventory</t>
         </is>
       </c>
-      <c r="C25" s="21">
-        <f>'Financial Data'!C23/'Financial Data'!$C$23*100</f>
-        <v/>
-      </c>
-      <c r="D25" s="21">
-        <f>'Financial Data'!D23/'Financial Data'!$C$23*100</f>
-        <v/>
-      </c>
-      <c r="E25" s="21">
-        <f>'Financial Data'!E23/'Financial Data'!$C$23*100</f>
-        <v/>
-      </c>
-      <c r="F25" s="21">
-        <f>'Financial Data'!F23/'Financial Data'!$C$23*100</f>
-        <v/>
-      </c>
-      <c r="G25" s="21">
-        <f>'Financial Data'!G23/'Financial Data'!$C$23*100</f>
-        <v/>
-      </c>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="21" t="n"/>
+      <c r="F25" s="21" t="n"/>
+      <c r="G25" s="21" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -2597,26 +1991,11 @@
           <t>Total Current Assets</t>
         </is>
       </c>
-      <c r="C26" s="21">
-        <f>'Financial Data'!C25/'Financial Data'!$C$25*100</f>
-        <v/>
-      </c>
-      <c r="D26" s="21">
-        <f>'Financial Data'!D25/'Financial Data'!$C$25*100</f>
-        <v/>
-      </c>
-      <c r="E26" s="21">
-        <f>'Financial Data'!E25/'Financial Data'!$C$25*100</f>
-        <v/>
-      </c>
-      <c r="F26" s="21">
-        <f>'Financial Data'!F25/'Financial Data'!$C$25*100</f>
-        <v/>
-      </c>
-      <c r="G26" s="21">
-        <f>'Financial Data'!G25/'Financial Data'!$C$25*100</f>
-        <v/>
-      </c>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="21" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -2624,26 +2003,11 @@
           <t>Total Assets</t>
         </is>
       </c>
-      <c r="C27" s="21">
-        <f>'Financial Data'!C29/'Financial Data'!$C$29*100</f>
-        <v/>
-      </c>
-      <c r="D27" s="21">
-        <f>'Financial Data'!D29/'Financial Data'!$C$29*100</f>
-        <v/>
-      </c>
-      <c r="E27" s="21">
-        <f>'Financial Data'!E29/'Financial Data'!$C$29*100</f>
-        <v/>
-      </c>
-      <c r="F27" s="21">
-        <f>'Financial Data'!F29/'Financial Data'!$C$29*100</f>
-        <v/>
-      </c>
-      <c r="G27" s="21">
-        <f>'Financial Data'!G29/'Financial Data'!$C$29*100</f>
-        <v/>
-      </c>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="21" t="n"/>
+      <c r="G27" s="21" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -2651,26 +2015,11 @@
           <t>Total Liabilities</t>
         </is>
       </c>
-      <c r="C28" s="21">
-        <f>'Financial Data'!C38/'Financial Data'!$C$38*100</f>
-        <v/>
-      </c>
-      <c r="D28" s="21">
-        <f>'Financial Data'!D38/'Financial Data'!$C$38*100</f>
-        <v/>
-      </c>
-      <c r="E28" s="21">
-        <f>'Financial Data'!E38/'Financial Data'!$C$38*100</f>
-        <v/>
-      </c>
-      <c r="F28" s="21">
-        <f>'Financial Data'!F38/'Financial Data'!$C$38*100</f>
-        <v/>
-      </c>
-      <c r="G28" s="21">
-        <f>'Financial Data'!G38/'Financial Data'!$C$38*100</f>
-        <v/>
-      </c>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="21" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -2678,26 +2027,11 @@
           <t>Total Shareholders' Equity</t>
         </is>
       </c>
-      <c r="C29" s="21">
-        <f>'Financial Data'!C39/'Financial Data'!$C$39*100</f>
-        <v/>
-      </c>
-      <c r="D29" s="21">
-        <f>'Financial Data'!D39/'Financial Data'!$C$39*100</f>
-        <v/>
-      </c>
-      <c r="E29" s="21">
-        <f>'Financial Data'!E39/'Financial Data'!$C$39*100</f>
-        <v/>
-      </c>
-      <c r="F29" s="21">
-        <f>'Financial Data'!F39/'Financial Data'!$C$39*100</f>
-        <v/>
-      </c>
-      <c r="G29" s="21">
-        <f>'Financial Data'!G39/'Financial Data'!$C$39*100</f>
-        <v/>
-      </c>
+      <c r="C29" s="21" t="n"/>
+      <c r="D29" s="21" t="n"/>
+      <c r="E29" s="21" t="n"/>
+      <c r="F29" s="21" t="n"/>
+      <c r="G29" s="21" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2786,26 +2120,11 @@
           <t>Current Ratio</t>
         </is>
       </c>
-      <c r="C10" s="22">
-        <f>'Financial Data'!C25/'Financial Data'!C35</f>
-        <v/>
-      </c>
-      <c r="D10" s="22">
-        <f>'Financial Data'!D25/'Financial Data'!D35</f>
-        <v/>
-      </c>
-      <c r="E10" s="22">
-        <f>'Financial Data'!E25/'Financial Data'!E35</f>
-        <v/>
-      </c>
-      <c r="F10" s="22">
-        <f>'Financial Data'!F25/'Financial Data'!F35</f>
-        <v/>
-      </c>
-      <c r="G10" s="22">
-        <f>'Financial Data'!G25/'Financial Data'!G35</f>
-        <v/>
-      </c>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="22" t="n"/>
+      <c r="G10" s="22" t="n"/>
       <c r="I10" s="23" t="inlineStr">
         <is>
           <t>Total Current Assets / Total Current Liabilities</t>
@@ -2818,26 +2137,11 @@
           <t>Quick Ratio</t>
         </is>
       </c>
-      <c r="C11" s="22">
-        <f>('Financial Data'!C25-'Financial Data'!C23)/'Financial Data'!C35</f>
-        <v/>
-      </c>
-      <c r="D11" s="22">
-        <f>('Financial Data'!D25-'Financial Data'!D23)/'Financial Data'!D35</f>
-        <v/>
-      </c>
-      <c r="E11" s="22">
-        <f>('Financial Data'!E25-'Financial Data'!E23)/'Financial Data'!E35</f>
-        <v/>
-      </c>
-      <c r="F11" s="22">
-        <f>('Financial Data'!F25-'Financial Data'!F23)/'Financial Data'!F35</f>
-        <v/>
-      </c>
-      <c r="G11" s="22">
-        <f>('Financial Data'!G25-'Financial Data'!G23)/'Financial Data'!G35</f>
-        <v/>
-      </c>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="22" t="n"/>
       <c r="I11" s="23" t="inlineStr">
         <is>
           <t>(Total Current Assets - Inventory) / Total Current Liabilities</t>
@@ -2850,26 +2154,11 @@
           <t>Cash Ratio</t>
         </is>
       </c>
-      <c r="C12" s="22">
-        <f>'Financial Data'!C21/'Financial Data'!C35</f>
-        <v/>
-      </c>
-      <c r="D12" s="22">
-        <f>'Financial Data'!D21/'Financial Data'!D35</f>
-        <v/>
-      </c>
-      <c r="E12" s="22">
-        <f>'Financial Data'!E21/'Financial Data'!E35</f>
-        <v/>
-      </c>
-      <c r="F12" s="22">
-        <f>'Financial Data'!F21/'Financial Data'!F35</f>
-        <v/>
-      </c>
-      <c r="G12" s="22">
-        <f>'Financial Data'!G21/'Financial Data'!G35</f>
-        <v/>
-      </c>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="22" t="n"/>
+      <c r="G12" s="22" t="n"/>
       <c r="I12" s="23" t="inlineStr">
         <is>
           <t>Cash &amp; Short-Term Investments / Total Current Liabilities</t>
@@ -2889,26 +2178,11 @@
           <t>Debt Ratio</t>
         </is>
       </c>
-      <c r="C15" s="16">
-        <f>'Financial Data'!C38/'Financial Data'!C29</f>
-        <v/>
-      </c>
-      <c r="D15" s="16">
-        <f>'Financial Data'!D38/'Financial Data'!D29</f>
-        <v/>
-      </c>
-      <c r="E15" s="16">
-        <f>'Financial Data'!E38/'Financial Data'!E29</f>
-        <v/>
-      </c>
-      <c r="F15" s="16">
-        <f>'Financial Data'!F38/'Financial Data'!F29</f>
-        <v/>
-      </c>
-      <c r="G15" s="16">
-        <f>'Financial Data'!G38/'Financial Data'!G29</f>
-        <v/>
-      </c>
+      <c r="C15" s="16" t="n"/>
+      <c r="D15" s="16" t="n"/>
+      <c r="E15" s="16" t="n"/>
+      <c r="F15" s="16" t="n"/>
+      <c r="G15" s="16" t="n"/>
       <c r="I15" s="23" t="inlineStr">
         <is>
           <t>Total Liabilities / Total Assets</t>
@@ -2921,26 +2195,11 @@
           <t>Debt-to-Equity</t>
         </is>
       </c>
-      <c r="C16" s="22">
-        <f>'Financial Data'!C38/'Financial Data'!C39</f>
-        <v/>
-      </c>
-      <c r="D16" s="22">
-        <f>'Financial Data'!D38/'Financial Data'!D39</f>
-        <v/>
-      </c>
-      <c r="E16" s="22">
-        <f>'Financial Data'!E38/'Financial Data'!E39</f>
-        <v/>
-      </c>
-      <c r="F16" s="22">
-        <f>'Financial Data'!F38/'Financial Data'!F39</f>
-        <v/>
-      </c>
-      <c r="G16" s="22">
-        <f>'Financial Data'!G38/'Financial Data'!G39</f>
-        <v/>
-      </c>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="22" t="n"/>
+      <c r="F16" s="22" t="n"/>
+      <c r="G16" s="22" t="n"/>
       <c r="I16" s="23" t="inlineStr">
         <is>
           <t>Total Liabilities / Total Shareholders' Equity</t>
@@ -2953,26 +2212,11 @@
           <t>Equity Multiplier</t>
         </is>
       </c>
-      <c r="C17" s="22">
-        <f>'Financial Data'!C29/'Financial Data'!C39</f>
-        <v/>
-      </c>
-      <c r="D17" s="22">
-        <f>'Financial Data'!D29/'Financial Data'!D39</f>
-        <v/>
-      </c>
-      <c r="E17" s="22">
-        <f>'Financial Data'!E29/'Financial Data'!E39</f>
-        <v/>
-      </c>
-      <c r="F17" s="22">
-        <f>'Financial Data'!F29/'Financial Data'!F39</f>
-        <v/>
-      </c>
-      <c r="G17" s="22">
-        <f>'Financial Data'!G29/'Financial Data'!G39</f>
-        <v/>
-      </c>
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="22" t="n"/>
+      <c r="F17" s="22" t="n"/>
+      <c r="G17" s="22" t="n"/>
       <c r="I17" s="23" t="inlineStr">
         <is>
           <t>Total Assets / Total Shareholders' Equity</t>
@@ -2985,26 +2229,11 @@
           <t>Times Interest Earned</t>
         </is>
       </c>
-      <c r="C18" s="22">
-        <f>'Financial Data'!C14/'Financial Data'!C15</f>
-        <v/>
-      </c>
-      <c r="D18" s="22">
-        <f>'Financial Data'!D14/'Financial Data'!D15</f>
-        <v/>
-      </c>
-      <c r="E18" s="22">
-        <f>'Financial Data'!E14/'Financial Data'!E15</f>
-        <v/>
-      </c>
-      <c r="F18" s="22">
-        <f>'Financial Data'!F14/'Financial Data'!F15</f>
-        <v/>
-      </c>
-      <c r="G18" s="22">
-        <f>'Financial Data'!G14/'Financial Data'!G15</f>
-        <v/>
-      </c>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="22" t="n"/>
+      <c r="G18" s="22" t="n"/>
       <c r="I18" s="23" t="inlineStr">
         <is>
           <t>Operating Income (EBIT) / Interest Expense</t>
@@ -3024,26 +2253,11 @@
           <t>Gross Margin</t>
         </is>
       </c>
-      <c r="C21" s="16">
-        <f>'Financial Data'!C12/'Financial Data'!C10</f>
-        <v/>
-      </c>
-      <c r="D21" s="16">
-        <f>'Financial Data'!D12/'Financial Data'!D10</f>
-        <v/>
-      </c>
-      <c r="E21" s="16">
-        <f>'Financial Data'!E12/'Financial Data'!E10</f>
-        <v/>
-      </c>
-      <c r="F21" s="16">
-        <f>'Financial Data'!F12/'Financial Data'!F10</f>
-        <v/>
-      </c>
-      <c r="G21" s="16">
-        <f>'Financial Data'!G12/'Financial Data'!G10</f>
-        <v/>
-      </c>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="16" t="n"/>
+      <c r="G21" s="16" t="n"/>
       <c r="I21" s="23" t="inlineStr">
         <is>
           <t>Gross Profit / Revenue</t>
@@ -3056,26 +2270,11 @@
           <t>Operating Margin</t>
         </is>
       </c>
-      <c r="C22" s="16">
-        <f>'Financial Data'!C14/'Financial Data'!C10</f>
-        <v/>
-      </c>
-      <c r="D22" s="16">
-        <f>'Financial Data'!D14/'Financial Data'!D10</f>
-        <v/>
-      </c>
-      <c r="E22" s="16">
-        <f>'Financial Data'!E14/'Financial Data'!E10</f>
-        <v/>
-      </c>
-      <c r="F22" s="16">
-        <f>'Financial Data'!F14/'Financial Data'!F10</f>
-        <v/>
-      </c>
-      <c r="G22" s="16">
-        <f>'Financial Data'!G14/'Financial Data'!G10</f>
-        <v/>
-      </c>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="n"/>
+      <c r="G22" s="16" t="n"/>
       <c r="I22" s="23" t="inlineStr">
         <is>
           <t>Operating Income (EBIT) / Revenue</t>
@@ -3088,26 +2287,11 @@
           <t>Net Profit Margin</t>
         </is>
       </c>
-      <c r="C23" s="16">
-        <f>'Financial Data'!C18/'Financial Data'!C10</f>
-        <v/>
-      </c>
-      <c r="D23" s="16">
-        <f>'Financial Data'!D18/'Financial Data'!D10</f>
-        <v/>
-      </c>
-      <c r="E23" s="16">
-        <f>'Financial Data'!E18/'Financial Data'!E10</f>
-        <v/>
-      </c>
-      <c r="F23" s="16">
-        <f>'Financial Data'!F18/'Financial Data'!F10</f>
-        <v/>
-      </c>
-      <c r="G23" s="16">
-        <f>'Financial Data'!G18/'Financial Data'!G10</f>
-        <v/>
-      </c>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="n"/>
+      <c r="G23" s="16" t="n"/>
       <c r="I23" s="23" t="inlineStr">
         <is>
           <t>Net Income / Revenue</t>
@@ -3120,26 +2304,11 @@
           <t>Return on Assets (ROA)</t>
         </is>
       </c>
-      <c r="C24" s="16">
-        <f>'Financial Data'!C18/'Financial Data'!C29</f>
-        <v/>
-      </c>
-      <c r="D24" s="16">
-        <f>'Financial Data'!D18/'Financial Data'!D29</f>
-        <v/>
-      </c>
-      <c r="E24" s="16">
-        <f>'Financial Data'!E18/'Financial Data'!E29</f>
-        <v/>
-      </c>
-      <c r="F24" s="16">
-        <f>'Financial Data'!F18/'Financial Data'!F29</f>
-        <v/>
-      </c>
-      <c r="G24" s="16">
-        <f>'Financial Data'!G18/'Financial Data'!G29</f>
-        <v/>
-      </c>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="16" t="n"/>
+      <c r="G24" s="16" t="n"/>
       <c r="I24" s="23" t="inlineStr">
         <is>
           <t>Net Income / Total Assets</t>
@@ -3152,26 +2321,11 @@
           <t>Return on Equity (ROE)</t>
         </is>
       </c>
-      <c r="C25" s="16">
-        <f>'Financial Data'!C18/'Financial Data'!C39</f>
-        <v/>
-      </c>
-      <c r="D25" s="16">
-        <f>'Financial Data'!D18/'Financial Data'!D39</f>
-        <v/>
-      </c>
-      <c r="E25" s="16">
-        <f>'Financial Data'!E18/'Financial Data'!E39</f>
-        <v/>
-      </c>
-      <c r="F25" s="16">
-        <f>'Financial Data'!F18/'Financial Data'!F39</f>
-        <v/>
-      </c>
-      <c r="G25" s="16">
-        <f>'Financial Data'!G18/'Financial Data'!G39</f>
-        <v/>
-      </c>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="16" t="n"/>
+      <c r="G25" s="16" t="n"/>
       <c r="I25" s="23" t="inlineStr">
         <is>
           <t>Net Income / Total Shareholders' Equity</t>
@@ -3191,26 +2345,11 @@
           <t>Inventory Turnover</t>
         </is>
       </c>
-      <c r="C28" s="22">
-        <f>'Financial Data'!C11/'Financial Data'!C23</f>
-        <v/>
-      </c>
-      <c r="D28" s="22">
-        <f>'Financial Data'!D11/'Financial Data'!D23</f>
-        <v/>
-      </c>
-      <c r="E28" s="22">
-        <f>'Financial Data'!E11/'Financial Data'!E23</f>
-        <v/>
-      </c>
-      <c r="F28" s="22">
-        <f>'Financial Data'!F11/'Financial Data'!F23</f>
-        <v/>
-      </c>
-      <c r="G28" s="22">
-        <f>'Financial Data'!G11/'Financial Data'!G23</f>
-        <v/>
-      </c>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="22" t="n"/>
+      <c r="F28" s="22" t="n"/>
+      <c r="G28" s="22" t="n"/>
       <c r="I28" s="23" t="inlineStr">
         <is>
           <t>Cost of Revenue (COGS) / Inventory</t>
@@ -3223,26 +2362,11 @@
           <t>Total Asset Turnover</t>
         </is>
       </c>
-      <c r="C29" s="22">
-        <f>'Financial Data'!C10/'Financial Data'!C29</f>
-        <v/>
-      </c>
-      <c r="D29" s="22">
-        <f>'Financial Data'!D10/'Financial Data'!D29</f>
-        <v/>
-      </c>
-      <c r="E29" s="22">
-        <f>'Financial Data'!E10/'Financial Data'!E29</f>
-        <v/>
-      </c>
-      <c r="F29" s="22">
-        <f>'Financial Data'!F10/'Financial Data'!F29</f>
-        <v/>
-      </c>
-      <c r="G29" s="22">
-        <f>'Financial Data'!G10/'Financial Data'!G29</f>
-        <v/>
-      </c>
+      <c r="C29" s="22" t="n"/>
+      <c r="D29" s="22" t="n"/>
+      <c r="E29" s="22" t="n"/>
+      <c r="F29" s="22" t="n"/>
+      <c r="G29" s="22" t="n"/>
       <c r="I29" s="23" t="inlineStr">
         <is>
           <t>Revenue / Total Assets</t>
@@ -3297,26 +2421,11 @@
           <t>Net Profit Margin</t>
         </is>
       </c>
-      <c r="C33" s="16">
-        <f>C23</f>
-        <v/>
-      </c>
-      <c r="D33" s="16">
-        <f>D23</f>
-        <v/>
-      </c>
-      <c r="E33" s="16">
-        <f>E23</f>
-        <v/>
-      </c>
-      <c r="F33" s="16">
-        <f>F23</f>
-        <v/>
-      </c>
-      <c r="G33" s="16">
-        <f>G23</f>
-        <v/>
-      </c>
+      <c r="C33" s="16" t="n"/>
+      <c r="D33" s="16" t="n"/>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="16" t="n"/>
+      <c r="G33" s="16" t="n"/>
       <c r="I33" s="24" t="inlineStr">
         <is>
           <t>pull it from the Profitability block above</t>
@@ -3329,26 +2438,11 @@
           <t>x  Total Asset Turnover</t>
         </is>
       </c>
-      <c r="C34" s="22">
-        <f>C29</f>
-        <v/>
-      </c>
-      <c r="D34" s="22">
-        <f>D29</f>
-        <v/>
-      </c>
-      <c r="E34" s="22">
-        <f>E29</f>
-        <v/>
-      </c>
-      <c r="F34" s="22">
-        <f>F29</f>
-        <v/>
-      </c>
-      <c r="G34" s="22">
-        <f>G29</f>
-        <v/>
-      </c>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n"/>
+      <c r="F34" s="22" t="n"/>
+      <c r="G34" s="22" t="n"/>
       <c r="I34" s="24" t="inlineStr">
         <is>
           <t>pull it from the Efficiency block above</t>
@@ -3361,26 +2455,11 @@
           <t>x  Equity Multiplier</t>
         </is>
       </c>
-      <c r="C35" s="22">
-        <f>C17</f>
-        <v/>
-      </c>
-      <c r="D35" s="22">
-        <f>D17</f>
-        <v/>
-      </c>
-      <c r="E35" s="22">
-        <f>E17</f>
-        <v/>
-      </c>
-      <c r="F35" s="22">
-        <f>F17</f>
-        <v/>
-      </c>
-      <c r="G35" s="22">
-        <f>G17</f>
-        <v/>
-      </c>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="22" t="n"/>
+      <c r="G35" s="22" t="n"/>
       <c r="I35" s="24" t="inlineStr">
         <is>
           <t>pull it from the Leverage block above</t>
@@ -3392,26 +2471,11 @@
         <f>  ROE (from DuPont)</f>
         <v/>
       </c>
-      <c r="C36" s="16">
-        <f>C33*C34*C35</f>
-        <v/>
-      </c>
-      <c r="D36" s="16">
-        <f>D33*D34*D35</f>
-        <v/>
-      </c>
-      <c r="E36" s="16">
-        <f>E33*E34*E35</f>
-        <v/>
-      </c>
-      <c r="F36" s="16">
-        <f>F33*F34*F35</f>
-        <v/>
-      </c>
-      <c r="G36" s="16">
-        <f>G33*G34*G35</f>
-        <v/>
-      </c>
+      <c r="C36" s="16" t="n"/>
+      <c r="D36" s="16" t="n"/>
+      <c r="E36" s="16" t="n"/>
+      <c r="F36" s="16" t="n"/>
+      <c r="G36" s="16" t="n"/>
       <c r="I36" s="24" t="inlineStr">
         <is>
           <t>multiply the three rows above</t>
@@ -3424,26 +2488,11 @@
           <t>ROE (from Profitability block)</t>
         </is>
       </c>
-      <c r="C37" s="16">
-        <f>C25</f>
-        <v/>
-      </c>
-      <c r="D37" s="16">
-        <f>D25</f>
-        <v/>
-      </c>
-      <c r="E37" s="16">
-        <f>E25</f>
-        <v/>
-      </c>
-      <c r="F37" s="16">
-        <f>F25</f>
-        <v/>
-      </c>
-      <c r="G37" s="16">
-        <f>G25</f>
-        <v/>
-      </c>
+      <c r="C37" s="16" t="n"/>
+      <c r="D37" s="16" t="n"/>
+      <c r="E37" s="16" t="n"/>
+      <c r="F37" s="16" t="n"/>
+      <c r="G37" s="16" t="n"/>
       <c r="I37" s="24" t="inlineStr">
         <is>
           <t>link to the ROE row above</t>
@@ -3456,26 +2505,11 @@
           <t>CHECK: difference</t>
         </is>
       </c>
-      <c r="C38" s="26">
-        <f>C36-C37</f>
-        <v/>
-      </c>
-      <c r="D38" s="26">
-        <f>D36-D37</f>
-        <v/>
-      </c>
-      <c r="E38" s="26">
-        <f>E36-E37</f>
-        <v/>
-      </c>
-      <c r="F38" s="26">
-        <f>F36-F37</f>
-        <v/>
-      </c>
-      <c r="G38" s="26">
-        <f>G36-G37</f>
-        <v/>
-      </c>
+      <c r="C38" s="26" t="n"/>
+      <c r="D38" s="26" t="n"/>
+      <c r="E38" s="26" t="n"/>
+      <c r="F38" s="26" t="n"/>
+      <c r="G38" s="26" t="n"/>
       <c r="I38" s="24" t="inlineStr">
         <is>
           <t>the two ROE rows minus each other - must be 0.00%</t>

</xml_diff>